<commit_message>
xlsx after the merge: argument modes of CHAR and CODE; the case books of the new and changed sets (arity, arrays, char-code, complex-text, date-noyear, lead-spaces, text-format, time-text) saved by Excel and read back, all as sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/xlsx/saved/arrays-3.xlsx
+++ b/test/excel/xlsx/saved/arrays-3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11004"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{662F3057-B3A1-0547-AF99-93C4395F820B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADB8EAA9-2494-8041-9124-B0A9313AE69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -804,6 +804,12 @@
     <t>lift:CEILING.PRECISE#2</t>
   </si>
   <si>
+    <t>lift:CHAR#1</t>
+  </si>
+  <si>
+    <t>lift:CHAR#2</t>
+  </si>
+  <si>
     <t>lift:CHIDIST#1</t>
   </si>
   <si>
@@ -912,6 +918,12 @@
     <t>lift:CLEAN#2</t>
   </si>
   <si>
+    <t>lift:CODE#1</t>
+  </si>
+  <si>
+    <t>lift:CODE#2</t>
+  </si>
+  <si>
     <t>lift:COMBIN#1</t>
   </si>
   <si>
@@ -1402,18 +1414,6 @@
   </si>
   <si>
     <t>lift:DB#6</t>
-  </si>
-  <si>
-    <t>lift:DB#7</t>
-  </si>
-  <si>
-    <t>lift:DB#8</t>
-  </si>
-  <si>
-    <t>lift:DB#9</t>
-  </si>
-  <si>
-    <t>lift:DB#10</t>
   </si>
   <si>
     <t>end</t>
@@ -7163,7 +7163,7 @@
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A197" ca="1">CHIDIST(D!B1:B2,10)</f>
+        <f t="array" aca="1" ref="A197" ca="1">CHAR(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B197">
@@ -7184,7 +7184,7 @@
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A198" ca="1">CHIDIST({1;2},10)</f>
+        <f t="array" aca="1" ref="A198" ca="1">CHAR({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B198">
@@ -7205,7 +7205,7 @@
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A199" ca="1">CHIDIST(18.307,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A199" ca="1">CHIDIST(D!B1:B2,10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B199">
@@ -7226,7 +7226,7 @@
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A200" ca="1">CHIDIST(18.307,{1;2})</f>
+        <f t="array" aca="1" ref="A200" ca="1">CHIDIST({1;2},10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B200">
@@ -7247,7 +7247,7 @@
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A201" ca="1">CHIINV(D!B1:B2,10)</f>
+        <f t="array" aca="1" ref="A201" ca="1">CHIDIST(18.307,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B201">
@@ -7268,7 +7268,7 @@
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A202" ca="1">CHIINV({1;2},10)</f>
+        <f t="array" aca="1" ref="A202" ca="1">CHIDIST(18.307,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B202">
@@ -7289,7 +7289,7 @@
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A203" ca="1">CHIINV(0.050001,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A203" ca="1">CHIINV(D!B1:B2,10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B203">
@@ -7310,7 +7310,7 @@
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A204" ca="1">CHIINV(0.050001,{1;2})</f>
+        <f t="array" aca="1" ref="A204" ca="1">CHIINV({1;2},10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B204">
@@ -7331,7 +7331,7 @@
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A205" ca="1">_xlfn.CHISQ.DIST(D!B1:B2,1,TRUE)</f>
+        <f t="array" aca="1" ref="A205" ca="1">CHIINV(0.050001,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B205">
@@ -7352,7 +7352,7 @@
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A206" ca="1">_xlfn.CHISQ.DIST({1;2},1,TRUE)</f>
+        <f t="array" aca="1" ref="A206" ca="1">CHIINV(0.050001,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B206">
@@ -7373,7 +7373,7 @@
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A207" ca="1">_xlfn.CHISQ.DIST(0.5,D!B1:B2,TRUE)</f>
+        <f t="array" aca="1" ref="A207" ca="1">_xlfn.CHISQ.DIST(D!B1:B2,1,TRUE)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B207">
@@ -7394,7 +7394,7 @@
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A208" ca="1">_xlfn.CHISQ.DIST(0.5,{1;2},TRUE)</f>
+        <f t="array" aca="1" ref="A208" ca="1">_xlfn.CHISQ.DIST({1;2},1,TRUE)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B208">
@@ -7415,7 +7415,7 @@
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A209" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A209" ca="1">_xlfn.CHISQ.DIST(0.5,1,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A209" ca="1">_xlfn.CHISQ.DIST(0.5,D!B1:B2,TRUE)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B209">
@@ -7436,7 +7436,7 @@
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A210" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A210" ca="1">_xlfn.CHISQ.DIST(0.5,1,{1;2})</f>
+        <f t="array" aca="1" ref="A210" ca="1">_xlfn.CHISQ.DIST(0.5,{1;2},TRUE)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B210">
@@ -7457,7 +7457,7 @@
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A211" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A211" ca="1">_xlfn.CHISQ.DIST.RT(D!B1:B2,10)</f>
+        <f t="array" aca="1" ref="A211" ca="1">_xlfn.CHISQ.DIST(0.5,1,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B211">
@@ -7478,7 +7478,7 @@
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A212" ca="1">_xlfn.CHISQ.DIST.RT({1;2},10)</f>
+        <f t="array" aca="1" ref="A212" ca="1">_xlfn.CHISQ.DIST(0.5,1,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B212">
@@ -7499,7 +7499,7 @@
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A213" ca="1">_xlfn.CHISQ.DIST.RT(18.307,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A213" ca="1">_xlfn.CHISQ.DIST.RT(D!B1:B2,10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B213">
@@ -7520,7 +7520,7 @@
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A214" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A214" ca="1">_xlfn.CHISQ.DIST.RT(18.307,{1;2})</f>
+        <f t="array" aca="1" ref="A214" ca="1">_xlfn.CHISQ.DIST.RT({1;2},10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B214">
@@ -7541,7 +7541,7 @@
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A215" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A215" ca="1">_xlfn.CHISQ.INV(D!B1:B2,1)</f>
+        <f t="array" aca="1" ref="A215" ca="1">_xlfn.CHISQ.DIST.RT(18.307,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B215">
@@ -7562,7 +7562,7 @@
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A216" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A216" ca="1">_xlfn.CHISQ.INV({1;2},1)</f>
+        <f t="array" aca="1" ref="A216" ca="1">_xlfn.CHISQ.DIST.RT(18.307,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B216">
@@ -7583,7 +7583,7 @@
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A217" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A217" ca="1">_xlfn.CHISQ.INV(0.93,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A217" ca="1">_xlfn.CHISQ.INV(D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B217">
@@ -7604,7 +7604,7 @@
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A218" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A218" ca="1">_xlfn.CHISQ.INV(0.93,{1;2})</f>
+        <f t="array" aca="1" ref="A218" ca="1">_xlfn.CHISQ.INV({1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B218">
@@ -7625,7 +7625,7 @@
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A219" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A219" ca="1">_xlfn.CHISQ.INV.RT(D!B1:B2,10)</f>
+        <f t="array" aca="1" ref="A219" ca="1">_xlfn.CHISQ.INV(0.93,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B219">
@@ -7646,7 +7646,7 @@
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A220" ca="1">_xlfn.CHISQ.INV.RT({1;2},10)</f>
+        <f t="array" aca="1" ref="A220" ca="1">_xlfn.CHISQ.INV(0.93,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B220">
@@ -7667,7 +7667,7 @@
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A221" ca="1">_xlfn.CHISQ.INV.RT(0.050001,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A221" ca="1">_xlfn.CHISQ.INV.RT(D!B1:B2,10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B221">
@@ -7688,7 +7688,7 @@
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A222" ca="1">_xlfn.CHISQ.INV.RT(0.050001,{1;2})</f>
+        <f t="array" aca="1" ref="A222" ca="1">_xlfn.CHISQ.INV.RT({1;2},10)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B222">
@@ -7709,7 +7709,7 @@
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A223" ca="1">CHOOSE(D!B1:B2,"a","b","c")</f>
+        <f t="array" aca="1" ref="A223" ca="1">_xlfn.CHISQ.INV.RT(0.050001,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B223">
@@ -7730,7 +7730,7 @@
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A224" ca="1">CHOOSE({1;2},"a","b","c")</f>
+        <f t="array" aca="1" ref="A224" ca="1">_xlfn.CHISQ.INV.RT(0.050001,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B224">
@@ -7750,176 +7750,176 @@
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A225" t="str" cm="1">
-        <f t="array" ref="A225">CHOOSE(2,D!B1:B2,"b","c")</f>
+      <c r="A225" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A225" ca="1">CHOOSE(D!B1:B2,"a","b","c")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B225">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C225">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D225" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E225" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A226" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A226" ca="1">CHOOSE({1;2},"a","b","c")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B226">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C226">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D226" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E226" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A227" t="str" cm="1">
+        <f t="array" ref="A227">CHOOSE(2,D!B1:B2,"b","c")</f>
         <v>b</v>
       </c>
-      <c r="B225">
+      <c r="B227">
         <f t="shared" si="9"/>
         <v>-3</v>
       </c>
-      <c r="C225">
+      <c r="C227">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="D225" t="str">
+      <c r="D227" t="str">
         <f t="shared" si="11"/>
         <v>b</v>
       </c>
-      <c r="E225" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A226" t="str" cm="1">
-        <f t="array" ref="A226">CHOOSE(2,{1;2},"b","c")</f>
+      <c r="E227" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A228" t="str" cm="1">
+        <f t="array" ref="A228">CHOOSE(2,{1;2},"b","c")</f>
         <v>b</v>
       </c>
-      <c r="B226">
+      <c r="B228">
         <f t="shared" si="9"/>
         <v>-3</v>
       </c>
-      <c r="C226">
+      <c r="C228">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="D226" t="str">
+      <c r="D228" t="str">
         <f t="shared" si="11"/>
         <v>b</v>
       </c>
-      <c r="E226" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A227" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A227" ca="1">CHOOSE(2,"a",D!B1:B2,"c")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B227">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
-      </c>
-      <c r="C227">
-        <f t="shared" ca="1" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D227" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="E227" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A228" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A228" ca="1">CHOOSE(2,"a",{1;2},"c")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B228">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
-      </c>
-      <c r="C228">
-        <f t="shared" ca="1" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D228" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
       <c r="E228" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A229" t="str" cm="1">
-        <f t="array" ref="A229">CHOOSE(2,"a","b",D!B1:B2)</f>
+      <c r="A229" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A229" ca="1">CHOOSE(2,"a",D!B1:B2,"c")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B229">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C229">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D229" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E229" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A230" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A230" ca="1">CHOOSE(2,"a",{1;2},"c")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B230">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C230">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D230" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E230" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A231" t="str" cm="1">
+        <f t="array" ref="A231">CHOOSE(2,"a","b",D!B1:B2)</f>
         <v>b</v>
       </c>
-      <c r="B229">
+      <c r="B231">
         <f t="shared" si="9"/>
         <v>-3</v>
       </c>
-      <c r="C229">
+      <c r="C231">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="D229" t="str">
+      <c r="D231" t="str">
         <f t="shared" si="11"/>
         <v>b</v>
       </c>
-      <c r="E229" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A230" t="str" cm="1">
-        <f t="array" ref="A230">CHOOSE(2,"a","b",{1;2})</f>
+      <c r="E231" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A232" t="str" cm="1">
+        <f t="array" ref="A232">CHOOSE(2,"a","b",{1;2})</f>
         <v>b</v>
       </c>
-      <c r="B230">
+      <c r="B232">
         <f t="shared" si="9"/>
         <v>-3</v>
       </c>
-      <c r="C230">
+      <c r="C232">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="D230" t="str">
+      <c r="D232" t="str">
         <f t="shared" si="11"/>
         <v>b</v>
       </c>
-      <c r="E230" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A231" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A231" ca="1">CLEAN(D!B1:B2)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B231">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
-      </c>
-      <c r="C231">
-        <f t="shared" ca="1" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D231" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="E231" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A232" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A232" ca="1">CLEAN({1;2})</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B232">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
-      </c>
-      <c r="C232">
-        <f t="shared" ca="1" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D232" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
       <c r="E232" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A233" ca="1">COMBIN(D!B1:B2,2)</f>
+        <f t="array" aca="1" ref="A233" ca="1">CLEAN(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B233">
@@ -7940,7 +7940,7 @@
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A234" ca="1">COMBIN({1;2},2)</f>
+        <f t="array" aca="1" ref="A234" ca="1">CLEAN({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B234">
@@ -7961,7 +7961,7 @@
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A235" ca="1">COMBIN(8,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A235" ca="1">CODE(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B235">
@@ -7982,7 +7982,7 @@
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A236" ca="1">COMBIN(8,{1;2})</f>
+        <f t="array" aca="1" ref="A236" ca="1">CODE({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B236">
@@ -8003,7 +8003,7 @@
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A237" ca="1">_xlfn.COMBINA(D!B1:B2,3)</f>
+        <f t="array" aca="1" ref="A237" ca="1">COMBIN(D!B1:B2,2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B237">
@@ -8024,7 +8024,7 @@
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A238" ca="1">_xlfn.COMBINA({1;2},3)</f>
+        <f t="array" aca="1" ref="A238" ca="1">COMBIN({1;2},2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B238">
@@ -8045,7 +8045,7 @@
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A239" ca="1">_xlfn.COMBINA(4,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A239" ca="1">COMBIN(8,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B239">
@@ -8066,7 +8066,7 @@
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A240" ca="1">_xlfn.COMBINA(4,{1;2})</f>
+        <f t="array" aca="1" ref="A240" ca="1">COMBIN(8,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B240">
@@ -8086,168 +8086,168 @@
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A241" t="e" cm="1">
-        <f t="array" ref="A241">COMPLEX(D!B1:B2,4)</f>
+      <c r="A241" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A241" ca="1">_xlfn.COMBINA(D!B1:B2,3)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B241">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C241">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D241" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E241" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A242" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A242" ca="1">_xlfn.COMBINA({1;2},3)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B242">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C242">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D242" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E242" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A243" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A243" ca="1">_xlfn.COMBINA(4,D!B1:B2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B243">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C243">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D243" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E243" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A244" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A244" ca="1">_xlfn.COMBINA(4,{1;2})</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B244">
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
+      </c>
+      <c r="C244">
+        <f t="shared" ca="1" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="D244" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+      <c r="E244" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A245" t="e" cm="1">
+        <f t="array" ref="A245">COMPLEX(D!B1:B2,4)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B245">
         <f t="shared" si="9"/>
         <v>3</v>
       </c>
-      <c r="C241">
+      <c r="C245">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="D241" t="str">
+      <c r="D245" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="E241" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A242" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A242" ca="1">COMPLEX({1;2},4)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B242">
+      <c r="E245" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A246" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A246" ca="1">COMPLEX({1;2},4)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B246">
         <f t="shared" ca="1" si="9"/>
         <v>9</v>
       </c>
-      <c r="C242">
+      <c r="C246">
         <f t="shared" ca="1" si="10"/>
         <v>0</v>
       </c>
-      <c r="D242" t="str">
+      <c r="D246" t="str">
         <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
-      <c r="E242" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A243" t="e" cm="1">
-        <f t="array" ref="A243">COMPLEX(3,D!B1:B2)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B243">
+      <c r="E246" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A247" t="e" cm="1">
+        <f t="array" ref="A247">COMPLEX(3,D!B1:B2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B247">
         <f t="shared" si="9"/>
         <v>3</v>
       </c>
-      <c r="C243">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D243" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="E243" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A244" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A244" ca="1">COMPLEX(3,{1;2})</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B244">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
-      </c>
-      <c r="C244">
-        <f t="shared" ca="1" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D244" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
-      </c>
-      <c r="E244" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A245" t="str" cm="1">
-        <f t="array" ref="A245">_xlfn.CONCAT(D!B1:B2,"b","c")</f>
-        <v>48bc</v>
-      </c>
-      <c r="B245">
-        <f t="shared" si="9"/>
-        <v>-3</v>
-      </c>
-      <c r="C245">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D245" t="str">
-        <f t="shared" si="11"/>
-        <v>48bc</v>
-      </c>
-      <c r="E245" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A246" t="str" cm="1">
-        <f t="array" ref="A246">_xlfn.CONCAT({1;2},"b","c")</f>
-        <v>12bc</v>
-      </c>
-      <c r="B246">
-        <f t="shared" si="9"/>
-        <v>-3</v>
-      </c>
-      <c r="C246">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="D246" t="str">
-        <f t="shared" si="11"/>
-        <v>12bc</v>
-      </c>
-      <c r="E246" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A247" t="str" cm="1">
-        <f t="array" ref="A247">_xlfn.CONCAT("a",D!B1:B2,"c")</f>
-        <v>a48c</v>
-      </c>
-      <c r="B247">
-        <f t="shared" si="9"/>
-        <v>-3</v>
-      </c>
       <c r="C247">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="D247" t="str">
         <f t="shared" si="11"/>
-        <v>a48c</v>
+        <v/>
       </c>
       <c r="E247" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A248" t="str" cm="1">
-        <f t="array" ref="A248">_xlfn.CONCAT("a",{1;2},"c")</f>
-        <v>a12c</v>
+      <c r="A248" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A248" ca="1">COMPLEX(3,{1;2})</f>
+        <v>#VALUE!</v>
       </c>
       <c r="B248">
-        <f t="shared" si="9"/>
-        <v>-3</v>
+        <f t="shared" ca="1" si="9"/>
+        <v>9</v>
       </c>
       <c r="C248">
-        <f t="shared" si="10"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0</v>
       </c>
       <c r="D248" t="str">
-        <f t="shared" si="11"/>
-        <v>a12c</v>
+        <f t="shared" ca="1" si="11"/>
+        <v/>
       </c>
       <c r="E248" t="s">
         <v>296</v>
@@ -8255,8 +8255,8 @@
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A249" t="str" cm="1">
-        <f t="array" ref="A249">_xlfn.CONCAT("a","b",D!B1:B2)</f>
-        <v>ab48</v>
+        <f t="array" ref="A249">_xlfn.CONCAT(D!B1:B2,"b","c")</f>
+        <v>48bc</v>
       </c>
       <c r="B249">
         <f t="shared" si="9"/>
@@ -8268,7 +8268,7 @@
       </c>
       <c r="D249" t="str">
         <f t="shared" si="11"/>
-        <v>ab48</v>
+        <v>48bc</v>
       </c>
       <c r="E249" t="s">
         <v>297</v>
@@ -8276,8 +8276,8 @@
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A250" t="str" cm="1">
-        <f t="array" ref="A250">_xlfn.CONCAT("a","b",{1;2})</f>
-        <v>ab12</v>
+        <f t="array" ref="A250">_xlfn.CONCAT({1;2},"b","c")</f>
+        <v>12bc</v>
       </c>
       <c r="B250">
         <f t="shared" si="9"/>
@@ -8289,91 +8289,91 @@
       </c>
       <c r="D250" t="str">
         <f t="shared" si="11"/>
-        <v>ab12</v>
+        <v>12bc</v>
       </c>
       <c r="E250" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="251" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A251" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A251" ca="1">CONCATENATE(D!B1:B2,"b")</f>
-        <v>#VALUE!</v>
+      <c r="A251" t="str" cm="1">
+        <f t="array" ref="A251">_xlfn.CONCAT("a",D!B1:B2,"c")</f>
+        <v>a48c</v>
       </c>
       <c r="B251">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
+        <f t="shared" si="9"/>
+        <v>-3</v>
       </c>
       <c r="C251">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="D251" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
+        <f t="shared" si="11"/>
+        <v>a48c</v>
       </c>
       <c r="E251" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A252" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A252" ca="1">CONCATENATE({1;2},"b")</f>
-        <v>#VALUE!</v>
+      <c r="A252" t="str" cm="1">
+        <f t="array" ref="A252">_xlfn.CONCAT("a",{1;2},"c")</f>
+        <v>a12c</v>
       </c>
       <c r="B252">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
+        <f t="shared" si="9"/>
+        <v>-3</v>
       </c>
       <c r="C252">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="D252" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
+        <f t="shared" si="11"/>
+        <v>a12c</v>
       </c>
       <c r="E252" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A253" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A253" ca="1">CONCATENATE("a",D!B1:B2)</f>
-        <v>#VALUE!</v>
+      <c r="A253" t="str" cm="1">
+        <f t="array" ref="A253">_xlfn.CONCAT("a","b",D!B1:B2)</f>
+        <v>ab48</v>
       </c>
       <c r="B253">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
+        <f t="shared" si="9"/>
+        <v>-3</v>
       </c>
       <c r="C253">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="D253" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
+        <f t="shared" si="11"/>
+        <v>ab48</v>
       </c>
       <c r="E253" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A254" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A254" ca="1">CONCATENATE("a",{1;2})</f>
-        <v>#VALUE!</v>
+      <c r="A254" t="str" cm="1">
+        <f t="array" ref="A254">_xlfn.CONCAT("a","b",{1;2})</f>
+        <v>ab12</v>
       </c>
       <c r="B254">
-        <f t="shared" ca="1" si="9"/>
-        <v>9</v>
+        <f t="shared" si="9"/>
+        <v>-3</v>
       </c>
       <c r="C254">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="D254" t="str">
-        <f t="shared" ca="1" si="11"/>
-        <v/>
+        <f t="shared" si="11"/>
+        <v>ab12</v>
       </c>
       <c r="E254" t="s">
         <v>302</v>
@@ -8381,7 +8381,7 @@
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A255" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A255" ca="1">CONFIDENCE(D!B1:B2,2.5,50)</f>
+        <f t="array" aca="1" ref="A255" ca="1">CONCATENATE(D!B1:B2,"b")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B255">
@@ -8402,7 +8402,7 @@
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A256" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A256" ca="1">CONFIDENCE({1;2},2.5,50)</f>
+        <f t="array" aca="1" ref="A256" ca="1">CONCATENATE({1;2},"b")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B256">
@@ -8423,7 +8423,7 @@
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A257" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A257" ca="1">CONFIDENCE(0.05,D!B1:B2,50)</f>
+        <f t="array" aca="1" ref="A257" ca="1">CONCATENATE("a",D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B257">
@@ -8444,7 +8444,7 @@
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A258" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A258" ca="1">CONFIDENCE(0.05,{1;2},50)</f>
+        <f t="array" aca="1" ref="A258" ca="1">CONCATENATE("a",{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B258">
@@ -8465,7 +8465,7 @@
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A259" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A259" ca="1">CONFIDENCE(0.05,2.5,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A259" ca="1">CONFIDENCE(D!B1:B2,2.5,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B259">
@@ -8486,7 +8486,7 @@
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A260" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A260" ca="1">CONFIDENCE(0.05,2.5,{1;2})</f>
+        <f t="array" aca="1" ref="A260" ca="1">CONFIDENCE({1;2},2.5,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B260">
@@ -8507,7 +8507,7 @@
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A261" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A261" ca="1">_xlfn.CONFIDENCE.NORM(D!B1:B2,2.5,50)</f>
+        <f t="array" aca="1" ref="A261" ca="1">CONFIDENCE(0.05,D!B1:B2,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B261">
@@ -8528,7 +8528,7 @@
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A262" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A262" ca="1">_xlfn.CONFIDENCE.NORM({1;2},2.5,50)</f>
+        <f t="array" aca="1" ref="A262" ca="1">CONFIDENCE(0.05,{1;2},50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B262">
@@ -8549,7 +8549,7 @@
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A263" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A263" ca="1">_xlfn.CONFIDENCE.NORM(0.05,D!B1:B2,50)</f>
+        <f t="array" aca="1" ref="A263" ca="1">CONFIDENCE(0.05,2.5,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B263">
@@ -8570,7 +8570,7 @@
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A264" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A264" ca="1">_xlfn.CONFIDENCE.NORM(0.05,{1;2},50)</f>
+        <f t="array" aca="1" ref="A264" ca="1">CONFIDENCE(0.05,2.5,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B264">
@@ -8591,7 +8591,7 @@
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A265" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A265" ca="1">_xlfn.CONFIDENCE.NORM(0.05,2.5,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A265" ca="1">_xlfn.CONFIDENCE.NORM(D!B1:B2,2.5,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B265">
@@ -8612,7 +8612,7 @@
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A266" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A266" ca="1">_xlfn.CONFIDENCE.NORM(0.05,2.5,{1;2})</f>
+        <f t="array" aca="1" ref="A266" ca="1">_xlfn.CONFIDENCE.NORM({1;2},2.5,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B266">
@@ -8633,7 +8633,7 @@
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A267" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A267" ca="1">_xlfn.CONFIDENCE.T(D!B1:B2,1,50)</f>
+        <f t="array" aca="1" ref="A267" ca="1">_xlfn.CONFIDENCE.NORM(0.05,D!B1:B2,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B267">
@@ -8654,7 +8654,7 @@
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A268" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A268" ca="1">_xlfn.CONFIDENCE.T({1;2},1,50)</f>
+        <f t="array" aca="1" ref="A268" ca="1">_xlfn.CONFIDENCE.NORM(0.05,{1;2},50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B268">
@@ -8675,7 +8675,7 @@
     </row>
     <row r="269" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A269" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A269" ca="1">_xlfn.CONFIDENCE.T(0.05,D!B1:B2,50)</f>
+        <f t="array" aca="1" ref="A269" ca="1">_xlfn.CONFIDENCE.NORM(0.05,2.5,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B269">
@@ -8696,7 +8696,7 @@
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A270" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A270" ca="1">_xlfn.CONFIDENCE.T(0.05,{1;2},50)</f>
+        <f t="array" aca="1" ref="A270" ca="1">_xlfn.CONFIDENCE.NORM(0.05,2.5,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B270">
@@ -8717,7 +8717,7 @@
     </row>
     <row r="271" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A271" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A271" ca="1">_xlfn.CONFIDENCE.T(0.05,1,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A271" ca="1">_xlfn.CONFIDENCE.T(D!B1:B2,1,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B271">
@@ -8738,7 +8738,7 @@
     </row>
     <row r="272" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A272" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A272" ca="1">_xlfn.CONFIDENCE.T(0.05,1,{1;2})</f>
+        <f t="array" aca="1" ref="A272" ca="1">_xlfn.CONFIDENCE.T({1;2},1,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B272">
@@ -8758,20 +8758,20 @@
       </c>
     </row>
     <row r="273" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A273" t="e" cm="1">
-        <f t="array" ref="A273">CONVERT(D!B1:B2,"lbm","kg")</f>
+      <c r="A273" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A273" ca="1">_xlfn.CONFIDENCE.T(0.05,D!B1:B2,50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B273">
-        <f t="shared" si="12"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>9</v>
       </c>
       <c r="C273">
-        <f t="shared" si="13"/>
+        <f t="shared" ca="1" si="13"/>
         <v>0</v>
       </c>
       <c r="D273" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ca="1" si="14"/>
         <v/>
       </c>
       <c r="E273" t="s">
@@ -8780,7 +8780,7 @@
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A274" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A274" ca="1">CONVERT({1;2},"lbm","kg")</f>
+        <f t="array" aca="1" ref="A274" ca="1">_xlfn.CONFIDENCE.T(0.05,{1;2},50)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B274">
@@ -8800,20 +8800,20 @@
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A275" t="e" cm="1">
-        <f t="array" ref="A275">CONVERT(1,D!B1:B2,"kg")</f>
+      <c r="A275" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A275" ca="1">_xlfn.CONFIDENCE.T(0.05,1,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B275">
-        <f t="shared" si="12"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>9</v>
       </c>
       <c r="C275">
-        <f t="shared" si="13"/>
+        <f t="shared" ca="1" si="13"/>
         <v>0</v>
       </c>
       <c r="D275" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ca="1" si="14"/>
         <v/>
       </c>
       <c r="E275" t="s">
@@ -8822,7 +8822,7 @@
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A276" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A276" ca="1">CONVERT(1,{1;2},"kg")</f>
+        <f t="array" aca="1" ref="A276" ca="1">_xlfn.CONFIDENCE.T(0.05,1,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B276">
@@ -8843,7 +8843,7 @@
     </row>
     <row r="277" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A277" t="e" cm="1">
-        <f t="array" ref="A277">CONVERT(1,"lbm",D!B1:B2)</f>
+        <f t="array" ref="A277">CONVERT(D!B1:B2,"lbm","kg")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B277">
@@ -8864,7 +8864,7 @@
     </row>
     <row r="278" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A278" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A278" ca="1">CONVERT(1,"lbm",{1;2})</f>
+        <f t="array" aca="1" ref="A278" ca="1">CONVERT({1;2},"lbm","kg")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B278">
@@ -8884,20 +8884,20 @@
       </c>
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A279" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A279" ca="1">COS(D!B1:B2)</f>
+      <c r="A279" t="e" cm="1">
+        <f t="array" ref="A279">CONVERT(1,D!B1:B2,"kg")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B279">
-        <f t="shared" ca="1" si="12"/>
-        <v>9</v>
+        <f t="shared" si="12"/>
+        <v>3</v>
       </c>
       <c r="C279">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="D279" t="str">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="E279" t="s">
@@ -8906,7 +8906,7 @@
     </row>
     <row r="280" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A280" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A280" ca="1">COS({1;2})</f>
+        <f t="array" aca="1" ref="A280" ca="1">CONVERT(1,{1;2},"kg")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B280">
@@ -8926,20 +8926,20 @@
       </c>
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A281" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A281" ca="1">COSH(D!B1:B2)</f>
+      <c r="A281" t="e" cm="1">
+        <f t="array" ref="A281">CONVERT(1,"lbm",D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B281">
-        <f t="shared" ca="1" si="12"/>
-        <v>9</v>
+        <f t="shared" si="12"/>
+        <v>3</v>
       </c>
       <c r="C281">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="D281" t="str">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="E281" t="s">
@@ -8948,7 +8948,7 @@
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A282" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A282" ca="1">COSH({1;2})</f>
+        <f t="array" aca="1" ref="A282" ca="1">CONVERT(1,"lbm",{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B282">
@@ -8969,7 +8969,7 @@
     </row>
     <row r="283" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A283" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A283" ca="1">_xlfn.COT(D!B1:B2)</f>
+        <f t="array" aca="1" ref="A283" ca="1">COS(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B283">
@@ -8990,7 +8990,7 @@
     </row>
     <row r="284" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A284" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A284" ca="1">_xlfn.COT({1;2})</f>
+        <f t="array" aca="1" ref="A284" ca="1">COS({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B284">
@@ -9011,7 +9011,7 @@
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A285" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A285" ca="1">_xlfn.COTH(D!B1:B2)</f>
+        <f t="array" aca="1" ref="A285" ca="1">COSH(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B285">
@@ -9032,7 +9032,7 @@
     </row>
     <row r="286" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A286" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A286" ca="1">_xlfn.COTH({1;2})</f>
+        <f t="array" aca="1" ref="A286" ca="1">COSH({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B286">
@@ -9053,7 +9053,7 @@
     </row>
     <row r="287" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A287" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A287" ca="1">COUNTIF(D!G1:G7,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A287" ca="1">_xlfn.COT(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B287">
@@ -9074,7 +9074,7 @@
     </row>
     <row r="288" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A288" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A288" ca="1">COUNTIF(D!G1:G7,{1;2})</f>
+        <f t="array" aca="1" ref="A288" ca="1">_xlfn.COT({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B288">
@@ -9095,7 +9095,7 @@
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A289" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A289" ca="1">COUNTIFS(D!G1:G7,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A289" ca="1">_xlfn.COTH(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B289">
@@ -9116,7 +9116,7 @@
     </row>
     <row r="290" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A290" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A290" ca="1">COUNTIFS(D!G1:G7,{1;2})</f>
+        <f t="array" aca="1" ref="A290" ca="1">_xlfn.COTH({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B290">
@@ -9136,20 +9136,20 @@
       </c>
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A291" t="e" cm="1">
-        <f t="array" ref="A291">COUPDAYBS(D!B1:B2,DATE(2011,11,15),2,1)</f>
+      <c r="A291" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A291" ca="1">COUNTIF(D!G1:G7,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B291">
-        <f t="shared" si="12"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>9</v>
       </c>
       <c r="C291">
-        <f t="shared" si="13"/>
+        <f t="shared" ca="1" si="13"/>
         <v>0</v>
       </c>
       <c r="D291" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ca="1" si="14"/>
         <v/>
       </c>
       <c r="E291" t="s">
@@ -9158,7 +9158,7 @@
     </row>
     <row r="292" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A292" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A292" ca="1">COUPDAYBS({1;2},DATE(2011,11,15),2,1)</f>
+        <f t="array" aca="1" ref="A292" ca="1">COUNTIF(D!G1:G7,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B292">
@@ -9178,20 +9178,20 @@
       </c>
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A293" t="e" cm="1">
-        <f t="array" ref="A293">COUPDAYBS(DATE(2011,1,25),D!B1:B2,2,1)</f>
+      <c r="A293" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A293" ca="1">COUNTIFS(D!G1:G7,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B293">
-        <f t="shared" si="12"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="12"/>
+        <v>9</v>
       </c>
       <c r="C293">
-        <f t="shared" si="13"/>
+        <f t="shared" ca="1" si="13"/>
         <v>0</v>
       </c>
       <c r="D293" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ca="1" si="14"/>
         <v/>
       </c>
       <c r="E293" t="s">
@@ -9200,7 +9200,7 @@
     </row>
     <row r="294" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A294" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A294" ca="1">COUPDAYBS(DATE(2011,1,25),{1;2},2,1)</f>
+        <f t="array" aca="1" ref="A294" ca="1">COUNTIFS(D!G1:G7,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B294">
@@ -9221,7 +9221,7 @@
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A295" t="e" cm="1">
-        <f t="array" ref="A295">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
+        <f t="array" ref="A295">COUPDAYBS(D!B1:B2,DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B295">
@@ -9242,7 +9242,7 @@
     </row>
     <row r="296" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A296" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A296" ca="1">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
+        <f t="array" aca="1" ref="A296" ca="1">COUPDAYBS({1;2},DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B296">
@@ -9263,7 +9263,7 @@
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A297" t="e" cm="1">
-        <f t="array" ref="A297">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
+        <f t="array" ref="A297">COUPDAYBS(DATE(2011,1,25),D!B1:B2,2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B297">
@@ -9284,7 +9284,7 @@
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A298" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A298" ca="1">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
+        <f t="array" aca="1" ref="A298" ca="1">COUPDAYBS(DATE(2011,1,25),{1;2},2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B298">
@@ -9305,7 +9305,7 @@
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A299" t="e" cm="1">
-        <f t="array" ref="A299">COUPDAYSNC(D!B1:B2,DATE(2011,11,15),2,1)</f>
+        <f t="array" ref="A299">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B299">
@@ -9326,7 +9326,7 @@
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A300" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A300" ca="1">COUPDAYSNC({1;2},DATE(2011,11,15),2,1)</f>
+        <f t="array" aca="1" ref="A300" ca="1">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B300">
@@ -9347,7 +9347,7 @@
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A301" t="e" cm="1">
-        <f t="array" ref="A301">COUPDAYSNC(DATE(2011,1,25),D!B1:B2,2,1)</f>
+        <f t="array" ref="A301">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B301">
@@ -9368,7 +9368,7 @@
     </row>
     <row r="302" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A302" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A302" ca="1">COUPDAYSNC(DATE(2011,1,25),{1;2},2,1)</f>
+        <f t="array" aca="1" ref="A302" ca="1">COUPDAYBS(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B302">
@@ -9389,7 +9389,7 @@
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A303" t="e" cm="1">
-        <f t="array" ref="A303">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
+        <f t="array" ref="A303">COUPDAYSNC(D!B1:B2,DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B303">
@@ -9410,7 +9410,7 @@
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A304" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A304" ca="1">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
+        <f t="array" aca="1" ref="A304" ca="1">COUPDAYSNC({1;2},DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B304">
@@ -9431,7 +9431,7 @@
     </row>
     <row r="305" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A305" t="e" cm="1">
-        <f t="array" ref="A305">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
+        <f t="array" ref="A305">COUPDAYSNC(DATE(2011,1,25),D!B1:B2,2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B305">
@@ -9452,7 +9452,7 @@
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A306" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A306" ca="1">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
+        <f t="array" aca="1" ref="A306" ca="1">COUPDAYSNC(DATE(2011,1,25),{1;2},2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B306">
@@ -9473,7 +9473,7 @@
     </row>
     <row r="307" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A307" t="e" cm="1">
-        <f t="array" ref="A307">COUPNCD(D!B1:B2,DATE(2011,11,15),2,1)</f>
+        <f t="array" ref="A307">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B307">
@@ -9494,7 +9494,7 @@
     </row>
     <row r="308" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A308" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A308" ca="1">COUPNCD({1;2},DATE(2011,11,15),2,1)</f>
+        <f t="array" aca="1" ref="A308" ca="1">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B308">
@@ -9515,7 +9515,7 @@
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A309" t="e" cm="1">
-        <f t="array" ref="A309">COUPNCD(DATE(2011,1,25),D!B1:B2,2,1)</f>
+        <f t="array" ref="A309">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B309">
@@ -9536,7 +9536,7 @@
     </row>
     <row r="310" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A310" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A310" ca="1">COUPNCD(DATE(2011,1,25),{1;2},2,1)</f>
+        <f t="array" aca="1" ref="A310" ca="1">COUPDAYSNC(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B310">
@@ -9557,7 +9557,7 @@
     </row>
     <row r="311" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A311" t="e" cm="1">
-        <f t="array" ref="A311">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
+        <f t="array" ref="A311">COUPNCD(D!B1:B2,DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B311">
@@ -9578,7 +9578,7 @@
     </row>
     <row r="312" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A312" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A312" ca="1">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
+        <f t="array" aca="1" ref="A312" ca="1">COUPNCD({1;2},DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B312">
@@ -9599,7 +9599,7 @@
     </row>
     <row r="313" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A313" t="e" cm="1">
-        <f t="array" ref="A313">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
+        <f t="array" ref="A313">COUPNCD(DATE(2011,1,25),D!B1:B2,2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B313">
@@ -9620,7 +9620,7 @@
     </row>
     <row r="314" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A314" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A314" ca="1">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
+        <f t="array" aca="1" ref="A314" ca="1">COUPNCD(DATE(2011,1,25),{1;2},2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B314">
@@ -9641,7 +9641,7 @@
     </row>
     <row r="315" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A315" t="e" cm="1">
-        <f t="array" ref="A315">COUPNUM(D!B1:B2,DATE(2011,11,15),2,1)</f>
+        <f t="array" ref="A315">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B315">
@@ -9662,7 +9662,7 @@
     </row>
     <row r="316" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A316" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A316" ca="1">COUPNUM({1;2},DATE(2011,11,15),2,1)</f>
+        <f t="array" aca="1" ref="A316" ca="1">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B316">
@@ -9683,7 +9683,7 @@
     </row>
     <row r="317" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A317" t="e" cm="1">
-        <f t="array" ref="A317">COUPNUM(DATE(2011,1,25),D!B1:B2,2,1)</f>
+        <f t="array" ref="A317">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B317">
@@ -9704,7 +9704,7 @@
     </row>
     <row r="318" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A318" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A318" ca="1">COUPNUM(DATE(2011,1,25),{1;2},2,1)</f>
+        <f t="array" aca="1" ref="A318" ca="1">COUPNCD(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B318">
@@ -9725,7 +9725,7 @@
     </row>
     <row r="319" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A319" t="e" cm="1">
-        <f t="array" ref="A319">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
+        <f t="array" ref="A319">COUPNUM(D!B1:B2,DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B319">
@@ -9746,7 +9746,7 @@
     </row>
     <row r="320" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A320" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A320" ca="1">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
+        <f t="array" aca="1" ref="A320" ca="1">COUPNUM({1;2},DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B320">
@@ -9767,7 +9767,7 @@
     </row>
     <row r="321" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A321" t="e" cm="1">
-        <f t="array" ref="A321">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
+        <f t="array" ref="A321">COUPNUM(DATE(2011,1,25),D!B1:B2,2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B321">
@@ -9788,7 +9788,7 @@
     </row>
     <row r="322" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A322" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A322" ca="1">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
+        <f t="array" aca="1" ref="A322" ca="1">COUPNUM(DATE(2011,1,25),{1;2},2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B322">
@@ -9809,7 +9809,7 @@
     </row>
     <row r="323" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A323" t="e" cm="1">
-        <f t="array" ref="A323">COUPPCD(D!B1:B2,DATE(2011,11,15),2,1)</f>
+        <f t="array" ref="A323">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B323">
@@ -9830,7 +9830,7 @@
     </row>
     <row r="324" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A324" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A324" ca="1">COUPPCD({1;2},DATE(2011,11,15),2,1)</f>
+        <f t="array" aca="1" ref="A324" ca="1">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B324">
@@ -9851,7 +9851,7 @@
     </row>
     <row r="325" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A325" t="e" cm="1">
-        <f t="array" ref="A325">COUPPCD(DATE(2011,1,25),D!B1:B2,2,1)</f>
+        <f t="array" ref="A325">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B325">
@@ -9872,7 +9872,7 @@
     </row>
     <row r="326" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A326" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A326" ca="1">COUPPCD(DATE(2011,1,25),{1;2},2,1)</f>
+        <f t="array" aca="1" ref="A326" ca="1">COUPNUM(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B326">
@@ -9893,7 +9893,7 @@
     </row>
     <row r="327" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A327" t="e" cm="1">
-        <f t="array" ref="A327">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
+        <f t="array" ref="A327">COUPPCD(D!B1:B2,DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B327">
@@ -9914,7 +9914,7 @@
     </row>
     <row r="328" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A328" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A328" ca="1">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
+        <f t="array" aca="1" ref="A328" ca="1">COUPPCD({1;2},DATE(2011,11,15),2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B328">
@@ -9935,7 +9935,7 @@
     </row>
     <row r="329" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A329" t="e" cm="1">
-        <f t="array" ref="A329">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
+        <f t="array" ref="A329">COUPPCD(DATE(2011,1,25),D!B1:B2,2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B329">
@@ -9956,7 +9956,7 @@
     </row>
     <row r="330" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A330" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A330" ca="1">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
+        <f t="array" aca="1" ref="A330" ca="1">COUPPCD(DATE(2011,1,25),{1;2},2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B330">
@@ -9976,20 +9976,20 @@
       </c>
     </row>
     <row r="331" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A331" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A331" ca="1">CRITBINOM(D!B1:B2,0.5,0.75)</f>
+      <c r="A331" t="e" cm="1">
+        <f t="array" ref="A331">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),D!B1:B2,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B331">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
+        <f t="shared" si="15"/>
+        <v>3</v>
       </c>
       <c r="C331">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="D331" t="str">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="E331" t="s">
@@ -9998,7 +9998,7 @@
     </row>
     <row r="332" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A332" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A332" ca="1">CRITBINOM({1;2},0.5,0.75)</f>
+        <f t="array" aca="1" ref="A332" ca="1">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),{1;2},1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B332">
@@ -10018,20 +10018,20 @@
       </c>
     </row>
     <row r="333" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A333" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A333" ca="1">CRITBINOM(6,D!B1:B2,0.75)</f>
+      <c r="A333" t="e" cm="1">
+        <f t="array" ref="A333">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),2,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B333">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
+        <f t="shared" si="15"/>
+        <v>3</v>
       </c>
       <c r="C333">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="D333" t="str">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="E333" t="s">
@@ -10040,7 +10040,7 @@
     </row>
     <row r="334" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A334" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A334" ca="1">CRITBINOM(6,{1;2},0.75)</f>
+        <f t="array" aca="1" ref="A334" ca="1">COUPPCD(DATE(2011,1,25),DATE(2011,11,15),2,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B334">
@@ -10061,7 +10061,7 @@
     </row>
     <row r="335" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A335" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A335" ca="1">CRITBINOM(6,0.5,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A335" ca="1">CRITBINOM(D!B1:B2,0.5,0.75)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B335">
@@ -10082,7 +10082,7 @@
     </row>
     <row r="336" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A336" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A336" ca="1">CRITBINOM(6,0.5,{1;2})</f>
+        <f t="array" aca="1" ref="A336" ca="1">CRITBINOM({1;2},0.5,0.75)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B336">
@@ -10103,7 +10103,7 @@
     </row>
     <row r="337" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A337" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A337" ca="1">_xlfn.CSC(D!B1:B2)</f>
+        <f t="array" aca="1" ref="A337" ca="1">CRITBINOM(6,D!B1:B2,0.75)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B337">
@@ -10124,7 +10124,7 @@
     </row>
     <row r="338" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A338" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A338" ca="1">_xlfn.CSC({1;2})</f>
+        <f t="array" aca="1" ref="A338" ca="1">CRITBINOM(6,{1;2},0.75)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B338">
@@ -10145,7 +10145,7 @@
     </row>
     <row r="339" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A339" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A339" ca="1">_xlfn.CSCH(D!B1:B2)</f>
+        <f t="array" aca="1" ref="A339" ca="1">CRITBINOM(6,0.5,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B339">
@@ -10166,7 +10166,7 @@
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A340" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A340" ca="1">_xlfn.CSCH({1;2})</f>
+        <f t="array" aca="1" ref="A340" ca="1">CRITBINOM(6,0.5,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B340">
@@ -10186,20 +10186,20 @@
       </c>
     </row>
     <row r="341" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A341" t="e" cm="1">
-        <f t="array" ref="A341">CUMIPMT(D!B1:B2,360,125000,13,24,0)</f>
+      <c r="A341" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A341" ca="1">_xlfn.CSC(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B341">
-        <f t="shared" si="15"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
       </c>
       <c r="C341">
-        <f t="shared" si="16"/>
+        <f t="shared" ca="1" si="16"/>
         <v>0</v>
       </c>
       <c r="D341" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" ca="1" si="17"/>
         <v/>
       </c>
       <c r="E341" t="s">
@@ -10208,7 +10208,7 @@
     </row>
     <row r="342" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A342" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A342" ca="1">CUMIPMT({1;2},360,125000,13,24,0)</f>
+        <f t="array" aca="1" ref="A342" ca="1">_xlfn.CSC({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B342">
@@ -10228,20 +10228,20 @@
       </c>
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A343" t="e" cm="1">
-        <f t="array" ref="A343">CUMIPMT(0.0075,D!B1:B2,125000,13,24,0)</f>
+      <c r="A343" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A343" ca="1">_xlfn.CSCH(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B343">
-        <f t="shared" si="15"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
       </c>
       <c r="C343">
-        <f t="shared" si="16"/>
+        <f t="shared" ca="1" si="16"/>
         <v>0</v>
       </c>
       <c r="D343" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" ca="1" si="17"/>
         <v/>
       </c>
       <c r="E343" t="s">
@@ -10250,7 +10250,7 @@
     </row>
     <row r="344" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A344" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A344" ca="1">CUMIPMT(0.0075,{1;2},125000,13,24,0)</f>
+        <f t="array" aca="1" ref="A344" ca="1">_xlfn.CSCH({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B344">
@@ -10271,7 +10271,7 @@
     </row>
     <row r="345" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A345" t="e" cm="1">
-        <f t="array" ref="A345">CUMIPMT(0.0075,360,D!B1:B2,13,24,0)</f>
+        <f t="array" ref="A345">CUMIPMT(D!B1:B2,360,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B345">
@@ -10292,7 +10292,7 @@
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A346" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A346" ca="1">CUMIPMT(0.0075,360,{1;2},13,24,0)</f>
+        <f t="array" aca="1" ref="A346" ca="1">CUMIPMT({1;2},360,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B346">
@@ -10313,7 +10313,7 @@
     </row>
     <row r="347" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A347" t="e" cm="1">
-        <f t="array" ref="A347">CUMIPMT(0.0075,360,125000,D!B1:B2,24,0)</f>
+        <f t="array" ref="A347">CUMIPMT(0.0075,D!B1:B2,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B347">
@@ -10334,7 +10334,7 @@
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A348" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A348" ca="1">CUMIPMT(0.0075,360,125000,{1;2},24,0)</f>
+        <f t="array" aca="1" ref="A348" ca="1">CUMIPMT(0.0075,{1;2},125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B348">
@@ -10355,7 +10355,7 @@
     </row>
     <row r="349" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A349" t="e" cm="1">
-        <f t="array" ref="A349">CUMIPMT(0.0075,360,125000,13,D!B1:B2,0)</f>
+        <f t="array" ref="A349">CUMIPMT(0.0075,360,D!B1:B2,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B349">
@@ -10376,7 +10376,7 @@
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A350" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A350" ca="1">CUMIPMT(0.0075,360,125000,13,{1;2},0)</f>
+        <f t="array" aca="1" ref="A350" ca="1">CUMIPMT(0.0075,360,{1;2},13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B350">
@@ -10397,7 +10397,7 @@
     </row>
     <row r="351" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A351" t="e" cm="1">
-        <f t="array" ref="A351">CUMIPMT(0.0075,360,125000,13,24,D!B1:B2)</f>
+        <f t="array" ref="A351">CUMIPMT(0.0075,360,125000,D!B1:B2,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B351">
@@ -10418,7 +10418,7 @@
     </row>
     <row r="352" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A352" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A352" ca="1">CUMIPMT(0.0075,360,125000,13,24,{1;2})</f>
+        <f t="array" aca="1" ref="A352" ca="1">CUMIPMT(0.0075,360,125000,{1;2},24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B352">
@@ -10439,7 +10439,7 @@
     </row>
     <row r="353" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A353" t="e" cm="1">
-        <f t="array" ref="A353">CUMPRINC(D!B1:B2,360,125000,13,24,0)</f>
+        <f t="array" ref="A353">CUMIPMT(0.0075,360,125000,13,D!B1:B2,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B353">
@@ -10460,7 +10460,7 @@
     </row>
     <row r="354" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A354" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A354" ca="1">CUMPRINC({1;2},360,125000,13,24,0)</f>
+        <f t="array" aca="1" ref="A354" ca="1">CUMIPMT(0.0075,360,125000,13,{1;2},0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B354">
@@ -10481,7 +10481,7 @@
     </row>
     <row r="355" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A355" t="e" cm="1">
-        <f t="array" ref="A355">CUMPRINC(0.0075,D!B1:B2,125000,13,24,0)</f>
+        <f t="array" ref="A355">CUMIPMT(0.0075,360,125000,13,24,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B355">
@@ -10502,7 +10502,7 @@
     </row>
     <row r="356" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A356" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A356" ca="1">CUMPRINC(0.0075,{1;2},125000,13,24,0)</f>
+        <f t="array" aca="1" ref="A356" ca="1">CUMIPMT(0.0075,360,125000,13,24,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B356">
@@ -10523,7 +10523,7 @@
     </row>
     <row r="357" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A357" t="e" cm="1">
-        <f t="array" ref="A357">CUMPRINC(0.0075,360,D!B1:B2,13,24,0)</f>
+        <f t="array" ref="A357">CUMPRINC(D!B1:B2,360,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B357">
@@ -10544,7 +10544,7 @@
     </row>
     <row r="358" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A358" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A358" ca="1">CUMPRINC(0.0075,360,{1;2},13,24,0)</f>
+        <f t="array" aca="1" ref="A358" ca="1">CUMPRINC({1;2},360,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B358">
@@ -10565,7 +10565,7 @@
     </row>
     <row r="359" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A359" t="e" cm="1">
-        <f t="array" ref="A359">CUMPRINC(0.0075,360,125000,D!B1:B2,24,0)</f>
+        <f t="array" ref="A359">CUMPRINC(0.0075,D!B1:B2,125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B359">
@@ -10586,7 +10586,7 @@
     </row>
     <row r="360" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A360" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A360" ca="1">CUMPRINC(0.0075,360,125000,{1;2},24,0)</f>
+        <f t="array" aca="1" ref="A360" ca="1">CUMPRINC(0.0075,{1;2},125000,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B360">
@@ -10607,7 +10607,7 @@
     </row>
     <row r="361" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A361" t="e" cm="1">
-        <f t="array" ref="A361">CUMPRINC(0.0075,360,125000,13,D!B1:B2,0)</f>
+        <f t="array" ref="A361">CUMPRINC(0.0075,360,D!B1:B2,13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B361">
@@ -10628,7 +10628,7 @@
     </row>
     <row r="362" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A362" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A362" ca="1">CUMPRINC(0.0075,360,125000,13,{1;2},0)</f>
+        <f t="array" aca="1" ref="A362" ca="1">CUMPRINC(0.0075,360,{1;2},13,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B362">
@@ -10649,7 +10649,7 @@
     </row>
     <row r="363" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A363" t="e" cm="1">
-        <f t="array" ref="A363">CUMPRINC(0.0075,360,125000,13,24,D!B1:B2)</f>
+        <f t="array" ref="A363">CUMPRINC(0.0075,360,125000,D!B1:B2,24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B363">
@@ -10670,7 +10670,7 @@
     </row>
     <row r="364" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A364" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A364" ca="1">CUMPRINC(0.0075,360,125000,13,24,{1;2})</f>
+        <f t="array" aca="1" ref="A364" ca="1">CUMPRINC(0.0075,360,125000,{1;2},24,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B364">
@@ -10690,20 +10690,20 @@
       </c>
     </row>
     <row r="365" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A365" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A365" ca="1">DATE(D!B1:B2,1,31)</f>
+      <c r="A365" t="e" cm="1">
+        <f t="array" ref="A365">CUMPRINC(0.0075,360,125000,13,D!B1:B2,0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B365">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
+        <f t="shared" si="15"/>
+        <v>3</v>
       </c>
       <c r="C365">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="D365" t="str">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="E365" t="s">
@@ -10712,7 +10712,7 @@
     </row>
     <row r="366" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A366" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A366" ca="1">DATE({1;2},1,31)</f>
+        <f t="array" aca="1" ref="A366" ca="1">CUMPRINC(0.0075,360,125000,13,{1;2},0)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B366">
@@ -10732,20 +10732,20 @@
       </c>
     </row>
     <row r="367" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A367" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A367" ca="1">DATE(2025,D!B1:B2,31)</f>
+      <c r="A367" t="e" cm="1">
+        <f t="array" ref="A367">CUMPRINC(0.0075,360,125000,13,24,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B367">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
+        <f t="shared" si="15"/>
+        <v>3</v>
       </c>
       <c r="C367">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="D367" t="str">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="E367" t="s">
@@ -10754,7 +10754,7 @@
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A368" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A368" ca="1">DATE(2025,{1;2},31)</f>
+        <f t="array" aca="1" ref="A368" ca="1">CUMPRINC(0.0075,360,125000,13,24,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B368">
@@ -10775,7 +10775,7 @@
     </row>
     <row r="369" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A369" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A369" ca="1">DATE(2025,1,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A369" ca="1">DATE(D!B1:B2,1,31)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B369">
@@ -10796,7 +10796,7 @@
     </row>
     <row r="370" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A370" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A370" ca="1">DATE(2025,1,{1;2})</f>
+        <f t="array" aca="1" ref="A370" ca="1">DATE({1;2},1,31)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B370">
@@ -10817,7 +10817,7 @@
     </row>
     <row r="371" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A371" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A371" ca="1">DATEDIF(D!B1:B2,37622,"Y")</f>
+        <f t="array" aca="1" ref="A371" ca="1">DATE(2025,D!B1:B2,31)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B371">
@@ -10838,7 +10838,7 @@
     </row>
     <row r="372" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A372" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A372" ca="1">DATEDIF({1;2},37622,"Y")</f>
+        <f t="array" aca="1" ref="A372" ca="1">DATE(2025,{1;2},31)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B372">
@@ -10859,7 +10859,7 @@
     </row>
     <row r="373" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A373" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A373" ca="1">DATEDIF(36892,D!B1:B2,"Y")</f>
+        <f t="array" aca="1" ref="A373" ca="1">DATE(2025,1,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B373">
@@ -10880,7 +10880,7 @@
     </row>
     <row r="374" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A374" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A374" ca="1">DATEDIF(36892,{1;2},"Y")</f>
+        <f t="array" aca="1" ref="A374" ca="1">DATE(2025,1,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B374">
@@ -10901,7 +10901,7 @@
     </row>
     <row r="375" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A375" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A375" ca="1">DATEDIF(36892,37622,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A375" ca="1">DATEDIF(D!B1:B2,37622,"Y")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B375">
@@ -10922,7 +10922,7 @@
     </row>
     <row r="376" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A376" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A376" ca="1">DATEDIF(36892,37622,{1;2})</f>
+        <f t="array" aca="1" ref="A376" ca="1">DATEDIF({1;2},37622,"Y")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B376">
@@ -10943,7 +10943,7 @@
     </row>
     <row r="377" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A377" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A377" ca="1">DATEVALUE(D!B1:B2)</f>
+        <f t="array" aca="1" ref="A377" ca="1">DATEDIF(36892,D!B1:B2,"Y")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B377">
@@ -10964,7 +10964,7 @@
     </row>
     <row r="378" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A378" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A378" ca="1">DATEVALUE({1;2})</f>
+        <f t="array" aca="1" ref="A378" ca="1">DATEDIF(36892,{1;2},"Y")</f>
         <v>#VALUE!</v>
       </c>
       <c r="B378">
@@ -10984,104 +10984,104 @@
       </c>
     </row>
     <row r="379" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A379" t="e" cm="1">
-        <f t="array" ref="A379">DAVERAGE(D!U1:Y7,D!B1:B2,D!AA1:AB2)</f>
+      <c r="A379" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A379" ca="1">DATEDIF(36892,37622,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B379">
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
+      </c>
+      <c r="C379">
+        <f t="shared" ca="1" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="D379" t="str">
+        <f t="shared" ca="1" si="17"/>
+        <v/>
+      </c>
+      <c r="E379" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="380" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A380" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A380" ca="1">DATEDIF(36892,37622,{1;2})</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B380">
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
+      </c>
+      <c r="C380">
+        <f t="shared" ca="1" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="D380" t="str">
+        <f t="shared" ca="1" si="17"/>
+        <v/>
+      </c>
+      <c r="E380" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="381" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A381" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A381" ca="1">DATEVALUE(D!B1:B2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B381">
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
+      </c>
+      <c r="C381">
+        <f t="shared" ca="1" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="D381" t="str">
+        <f t="shared" ca="1" si="17"/>
+        <v/>
+      </c>
+      <c r="E381" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="382" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A382" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="A382" ca="1">DATEVALUE({1;2})</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B382">
+        <f t="shared" ca="1" si="15"/>
+        <v>9</v>
+      </c>
+      <c r="C382">
+        <f t="shared" ca="1" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="D382" t="str">
+        <f t="shared" ca="1" si="17"/>
+        <v/>
+      </c>
+      <c r="E382" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="383" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A383" t="e" cm="1">
+        <f t="array" ref="A383">DAVERAGE(D!U1:Y7,D!B1:B2,D!AA1:AB2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B383">
         <f t="shared" si="15"/>
         <v>3</v>
       </c>
-      <c r="C379">
+      <c r="C383">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="D379" t="str">
+      <c r="D383" t="str">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="E379" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A380" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A380" ca="1">DAVERAGE(D!U1:Y7,{1;2},D!AA1:AB2)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B380">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
-      </c>
-      <c r="C380">
-        <f t="shared" ca="1" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="D380" t="str">
-        <f t="shared" ca="1" si="17"/>
-        <v/>
-      </c>
-      <c r="E380" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="381" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A381" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A381" ca="1">DAY(D!B1:B2)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B381">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
-      </c>
-      <c r="C381">
-        <f t="shared" ca="1" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="D381" t="str">
-        <f t="shared" ca="1" si="17"/>
-        <v/>
-      </c>
-      <c r="E381" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="382" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A382" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A382" ca="1">DAY({1;2})</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B382">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
-      </c>
-      <c r="C382">
-        <f t="shared" ca="1" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="D382" t="str">
-        <f t="shared" ca="1" si="17"/>
-        <v/>
-      </c>
-      <c r="E382" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="383" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A383" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A383" ca="1">_xlfn.DAYS(D!B1:B2,44228)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B383">
-        <f t="shared" ca="1" si="15"/>
-        <v>9</v>
-      </c>
-      <c r="C383">
-        <f t="shared" ca="1" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="D383" t="str">
-        <f t="shared" ca="1" si="17"/>
         <v/>
       </c>
       <c r="E383" t="s">
@@ -11090,7 +11090,7 @@
     </row>
     <row r="384" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A384" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A384" ca="1">_xlfn.DAYS({1;2},44228)</f>
+        <f t="array" aca="1" ref="A384" ca="1">DAVERAGE(D!U1:Y7,{1;2},D!AA1:AB2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B384">
@@ -11111,7 +11111,7 @@
     </row>
     <row r="385" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A385" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A385" ca="1">_xlfn.DAYS(44270,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A385" ca="1">DAY(D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B385">
@@ -11132,7 +11132,7 @@
     </row>
     <row r="386" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A386" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A386" ca="1">_xlfn.DAYS(44270,{1;2})</f>
+        <f t="array" aca="1" ref="A386" ca="1">DAY({1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B386">
@@ -11153,7 +11153,7 @@
     </row>
     <row r="387" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A387" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A387" ca="1">DAYS360(D!B1:B2,40908)</f>
+        <f t="array" aca="1" ref="A387" ca="1">_xlfn.DAYS(D!B1:B2,44228)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B387">
@@ -11174,7 +11174,7 @@
     </row>
     <row r="388" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A388" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A388" ca="1">DAYS360({1;2},40908)</f>
+        <f t="array" aca="1" ref="A388" ca="1">_xlfn.DAYS({1;2},44228)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B388">
@@ -11195,7 +11195,7 @@
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A389" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A389" ca="1">DAYS360(40573,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A389" ca="1">_xlfn.DAYS(44270,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B389">
@@ -11216,7 +11216,7 @@
     </row>
     <row r="390" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A390" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A390" ca="1">DAYS360(40573,{1;2})</f>
+        <f t="array" aca="1" ref="A390" ca="1">_xlfn.DAYS(44270,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B390">
@@ -11237,7 +11237,7 @@
     </row>
     <row r="391" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A391" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A391" ca="1">DB(D!B1:B2,100000,6,1,7)</f>
+        <f t="array" aca="1" ref="A391" ca="1">DAYS360(D!B1:B2,40908)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B391">
@@ -11258,7 +11258,7 @@
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A392" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A392" ca="1">DB({1;2},100000,6,1,7)</f>
+        <f t="array" aca="1" ref="A392" ca="1">DAYS360({1;2},40908)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B392">
@@ -11279,7 +11279,7 @@
     </row>
     <row r="393" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A393" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A393" ca="1">DB(1000000,D!B1:B2,6,1,7)</f>
+        <f t="array" aca="1" ref="A393" ca="1">DAYS360(40573,D!B1:B2)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B393">
@@ -11300,7 +11300,7 @@
     </row>
     <row r="394" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A394" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A394" ca="1">DB(1000000,{1;2},6,1,7)</f>
+        <f t="array" aca="1" ref="A394" ca="1">DAYS360(40573,{1;2})</f>
         <v>#VALUE!</v>
       </c>
       <c r="B394">
@@ -11321,7 +11321,7 @@
     </row>
     <row r="395" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A395" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A395" ca="1">DB(1000000,100000,D!B1:B2,1,7)</f>
+        <f t="array" aca="1" ref="A395" ca="1">DB(D!B1:B2,100000,6,1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B395">
@@ -11342,7 +11342,7 @@
     </row>
     <row r="396" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A396" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A396" ca="1">DB(1000000,100000,{1;2},1,7)</f>
+        <f t="array" aca="1" ref="A396" ca="1">DB({1;2},100000,6,1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B396">
@@ -11363,7 +11363,7 @@
     </row>
     <row r="397" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A397" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A397" ca="1">DB(1000000,100000,6,D!B1:B2,7)</f>
+        <f t="array" aca="1" ref="A397" ca="1">DB(1000000,D!B1:B2,6,1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B397">
@@ -11384,7 +11384,7 @@
     </row>
     <row r="398" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A398" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A398" ca="1">DB(1000000,100000,6,{1;2},7)</f>
+        <f t="array" aca="1" ref="A398" ca="1">DB(1000000,{1;2},6,1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B398">
@@ -11405,7 +11405,7 @@
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A399" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A399" ca="1">DB(1000000,100000,6,1,D!B1:B2)</f>
+        <f t="array" aca="1" ref="A399" ca="1">DB(1000000,100000,D!B1:B2,1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B399">
@@ -11426,7 +11426,7 @@
     </row>
     <row r="400" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A400" t="e" cm="1" vm="1">
-        <f t="array" aca="1" ref="A400" ca="1">DB(1000000,100000,6,1,{1;2})</f>
+        <f t="array" aca="1" ref="A400" ca="1">DB(1000000,100000,{1;2},1,7)</f>
         <v>#VALUE!</v>
       </c>
       <c r="B400">

</xml_diff>